<commit_message>
feat: Add announcement management functionality
- Implemented announcement creation, updating, publishing, and deletion in the backend.
- Added new API endpoints for announcements in the main application.
- Updated the database schema to include an announcements table.
- Enhanced the admin interface to manage announcements, including fields for title, content, and visibility.
- Integrated announcement management into the frontend, allowing users to create, edit, and publish announcements.
- Updated permission checks to include announcement management capabilities.
- Modified existing components to support new announcement features and styles.
</commit_message>
<xml_diff>
--- a/整改与实施计划表.xlsx
+++ b/整改与实施计划表.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/micropue/Desktop/前后端项目/虎虎校园跑登记系统/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33C97202-96DB-C344-A648-57BC22D6D613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E0303D3-AAD3-8E45-A07C-32524AC30C9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16980" xr2:uid="{9DB7FF6E-2683-AE40-AAEF-56B36CD941DB}"/>
+    <workbookView xWindow="2800" yWindow="600" windowWidth="29400" windowHeight="16960" xr2:uid="{9DB7FF6E-2683-AE40-AAEF-56B36CD941DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$18</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="52">
   <si>
     <t>编号</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -226,6 +229,22 @@
   </si>
   <si>
     <t>已完成</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在聊天界面自己的气泡加时间</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>实际完成时间</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>撤回消息</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>版本未更新时不允许访问</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -285,7 +304,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -308,13 +327,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -348,7 +380,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="58" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -744,7 +791,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D86C6A56-1155-254D-8306-53828F17833A}">
-  <dimension ref="A1:K15"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="29.83203125" style="1" customWidth="1"/>
@@ -752,9 +800,10 @@
     <col min="4" max="5" width="15.5" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
     <col min="11" max="11" width="12.5" customWidth="1"/>
+    <col min="12" max="12" width="14.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -788,8 +837,11 @@
       <c r="K1" s="5" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" ht="34">
+      <c r="L1" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="34" hidden="1">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -824,8 +876,11 @@
       <c r="K2" s="2" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" ht="34">
+      <c r="L2" s="12">
+        <v>46176</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="34" hidden="1">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -843,7 +898,7 @@
         <v>52</v>
       </c>
       <c r="G3" s="2">
-        <f t="shared" ref="G3:G14" si="0">F3-E3</f>
+        <f t="shared" ref="G3:G17" si="0">F3-E3</f>
         <v>-8</v>
       </c>
       <c r="H3" s="2" t="s">
@@ -858,8 +913,11 @@
       <c r="K3" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" ht="34">
+      <c r="L3" s="12">
+        <v>46176</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="34">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -892,8 +950,9 @@
       <c r="K4" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" ht="17">
+      <c r="L4" s="2"/>
+    </row>
+    <row r="5" spans="1:12" ht="17">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -928,8 +987,9 @@
       <c r="K5" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" ht="51">
+      <c r="L5" s="2"/>
+    </row>
+    <row r="6" spans="1:12" ht="51" hidden="1">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -962,8 +1022,9 @@
         <v>30</v>
       </c>
       <c r="K6" s="2"/>
-    </row>
-    <row r="7" spans="1:11" ht="34">
+      <c r="L6" s="2"/>
+    </row>
+    <row r="7" spans="1:12" ht="34">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -996,8 +1057,9 @@
       <c r="K7" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" ht="34">
+      <c r="L7" s="2"/>
+    </row>
+    <row r="8" spans="1:12" ht="34">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1030,8 +1092,9 @@
       <c r="K8" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" ht="17">
+      <c r="L8" s="2"/>
+    </row>
+    <row r="9" spans="1:12" ht="17" hidden="1">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1062,8 +1125,9 @@
         <v>30</v>
       </c>
       <c r="K9" s="2"/>
-    </row>
-    <row r="10" spans="1:11" ht="68">
+      <c r="L9" s="2"/>
+    </row>
+    <row r="10" spans="1:12" ht="68">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1098,8 +1162,9 @@
       <c r="K10" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" ht="34">
+      <c r="L10" s="2"/>
+    </row>
+    <row r="11" spans="1:12" ht="34">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1134,8 +1199,9 @@
       <c r="K11" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" ht="34">
+      <c r="L11" s="2"/>
+    </row>
+    <row r="12" spans="1:12" ht="34" hidden="1">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1166,8 +1232,9 @@
         <v>30</v>
       </c>
       <c r="K12" s="2"/>
-    </row>
-    <row r="13" spans="1:11" ht="17">
+      <c r="L12" s="2"/>
+    </row>
+    <row r="13" spans="1:12" ht="17" hidden="1">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1200,56 +1267,184 @@
       <c r="K13" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" s="7" customFormat="1">
-      <c r="A14" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E14" s="6">
-        <f>SUM(E2:E13)</f>
-        <v>633.20000000000005</v>
-      </c>
-      <c r="F14" s="4">
-        <f>SUM(F2:F13)</f>
-        <v>557</v>
+      <c r="L13" s="12">
+        <v>46176</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="17">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="2">
+        <v>0</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0</v>
       </c>
       <c r="G14" s="2">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="L14" s="2"/>
+    </row>
+    <row r="15" spans="1:12" ht="17" hidden="1">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="3"/>
+      <c r="D15" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="2">
+        <v>30</v>
+      </c>
+      <c r="F15" s="2">
+        <v>30</v>
+      </c>
+      <c r="G15" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="L15" s="2"/>
+    </row>
+    <row r="16" spans="1:12" ht="17">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" s="3"/>
+      <c r="D16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" s="2">
+        <v>0</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0</v>
+      </c>
+      <c r="G16" s="2">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="L16" s="2"/>
+    </row>
+    <row r="17" spans="1:12" s="7" customFormat="1" hidden="1">
+      <c r="A17" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E17" s="6">
+        <f>SUM(E2:E16)</f>
+        <v>663.2</v>
+      </c>
+      <c r="F17" s="4">
+        <f>SUM(F2:F16)</f>
+        <v>587</v>
+      </c>
+      <c r="G17" s="2">
+        <f t="shared" si="0"/>
         <v>-76.200000000000045</v>
       </c>
-      <c r="H14" s="9" t="s">
+      <c r="H17" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="I14" s="9"/>
-      <c r="J14" s="10">
-        <f>F14-SUMIF(I2:I12,"已支付",F2:F12)</f>
-        <v>350</v>
-      </c>
-      <c r="K14" s="10"/>
-    </row>
-    <row r="15" spans="1:11">
-      <c r="H15" s="10" t="s">
+      <c r="I17" s="9"/>
+      <c r="J17" s="10">
+        <f>F17-SUMIF(I2:I12,"已支付",F2:F12)</f>
+        <v>380</v>
+      </c>
+      <c r="K17" s="10"/>
+      <c r="L17" s="5"/>
+    </row>
+    <row r="18" spans="1:12" hidden="1">
+      <c r="A18" s="13"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="I15" s="11"/>
-      <c r="J15" s="10">
+      <c r="I18" s="16"/>
+      <c r="J18" s="15">
         <f>SUMIF(I2:I12,"已支付",F2:F12)</f>
         <v>207</v>
       </c>
-      <c r="K15" s="10"/>
+      <c r="K18" s="15"/>
+      <c r="L18" s="13"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:L18" xr:uid="{D86C6A56-1155-254D-8306-53828F17833A}">
+    <filterColumn colId="8">
+      <filters>
+        <filter val="已支付"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="9">
+      <filters>
+        <filter val="未完成"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="5">
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="J18:K18"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="E2:E1048576">
@@ -1268,7 +1463,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I1:I13 J14 I16:I1048576">
+  <conditionalFormatting sqref="I1:I16 J17 I19:I1048576">
     <cfRule type="cellIs" dxfId="2" priority="8" operator="equal">
       <formula>"已支付"</formula>
     </cfRule>

</xml_diff>